<commit_message>
DAT100-2773 - Modificación archivo base de tipo Acuerdo
Se modifica a texto las columnas de fecha
</commit_message>
<xml_diff>
--- a/WebDataAgro/Templates/AltaMasiva.xlsx
+++ b/WebDataAgro/Templates/AltaMasiva.xlsx
@@ -129,8 +129,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -212,7 +213,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -221,7 +222,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -243,15 +252,15 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr defaultColWidth="8.4609375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.4609375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="6.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="15.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="3.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11.99"/>
@@ -262,50 +271,50 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="9.42"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
DAT-920 Se corrije nombre de San Lorenzo en archivo de AltaMasiva
</commit_message>
<xml_diff>
--- a/WebDataAgro/Templates/AltaMasiva.xlsx
+++ b/WebDataAgro/Templates/AltaMasiva.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="AltaMasiva" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Data" sheetId="2" state="hidden" r:id="rId3"/>
+    <sheet name="AltaMasiva" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Data" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -83,7 +83,7 @@
     <t xml:space="preserve">x</t>
   </si>
   <si>
-    <t xml:space="preserve">S. Lorenzo</t>
+    <t xml:space="preserve">San Lorenzo</t>
   </si>
   <si>
     <t xml:space="preserve">Maiz</t>
@@ -246,13 +246,119 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr defaultColWidth="8.4609375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.4609375" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.57"/>
@@ -357,7 +463,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="8.4609375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.4609375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.99"/>

</xml_diff>